<commit_message>
APK 3.17.0: estados de mantenimiento y filtro unificados (Programado/Reprogramado/Finalizado)
</commit_message>
<xml_diff>
--- a/excel_ejemplo/mantenimientos.xlsx
+++ b/excel_ejemplo/mantenimientos.xlsx
@@ -70,12 +70,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Finalizado</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -112,7 +112,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Reprogramado</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -149,7 +149,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Realizado</t>
+          <t>Finalizado</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Programado</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -223,7 +223,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Programado</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -260,7 +260,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Programado</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">

</xml_diff>